<commit_message>
feat(xlsx): enhanced metadata, default values, and conditional rows
- Added comprehensive metadata markers: $year, $month, $day, $rowNumber, $rowIndex, $colNumber, $colIndex, $columnLetter, and parity markers for rows and columns.
- Implemented default value support using the `||` operator in interpolation paths.
- Added support for boolean-based conditional row rendering using `[[]]` markers.
- Refactored interpolation logic for better robustness and maintainability.
- Updated documentation and established the roadmap for @interpolator/markdown.
</commit_message>
<xml_diff>
--- a/packages/xlsx/tests/fixtures/result.xlsx
+++ b/packages/xlsx/tests/fixtures/result.xlsx
@@ -16,7 +16,7 @@
     <t>Name: Germán</t>
   </si>
   <si>
-    <t>Date: Mon Jan 01 2024 21:00:00 GMT-0300 (Argentina Standard Time)</t>
+    <t>Date: Tue Jan 02 2024 00:00:00 GMT+0000 (Coordinated Universal Time)</t>
   </si>
   <si>
     <t>ID: 001</t>
@@ -28,7 +28,7 @@
     <t>Price: 120.5</t>
   </si>
   <si>
-    <t>Item date: Tue Jan 02 2024 21:00:00 GMT-0300 (Argentina Standard Time)</t>
+    <t>Item date: Wed Jan 03 2024 00:00:00 GMT+0000 (Coordinated Universal Time)</t>
   </si>
   <si>
     <t>Missing: [[items.missingProp]]</t>
@@ -468,7 +468,7 @@
         <v>6</v>
       </c>
       <c r="F3">
-        <f>B2*C2</f>
+        <f>B3*C3</f>
       </c>
     </row>
   </sheetData>

</xml_diff>